<commit_message>
Add DDI survey and Safes roadmap activities
</commit_message>
<xml_diff>
--- a/Дорожные карты по повышению рейтинга DD.xlsx
+++ b/Дорожные карты по повышению рейтинга DD.xlsx
@@ -38026,7 +38026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M29"/>
+  <dimension ref="A1:M32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15.75"/>
   <cols>
     <col width="6.125" customWidth="1" style="181" min="1" max="1"/>
@@ -39390,6 +39390,112 @@
     </row>
     <row r="29" s="181">
       <c r="C29" s="383" t="n"/>
+    </row>
+    <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="30">
+      <c r="A30" s="70" t="str">
+        <v>Сейфы_Знание ключевых метрик</v>
+      </c>
+      <c r="B30" s="369" t="str">
+        <v>Сейфы</v>
+      </c>
+      <c r="C30" s="327" t="str">
+        <v>Q42026</v>
+      </c>
+      <c r="D30" s="370" t="str">
+        <v>Знание ключевых метрик</v>
+      </c>
+      <c r="E30" s="371" t="str">
+        <v>Валидация данных об Объеме целевого рынка в России, объем целевого рынка в Сбере, клиенты с продуктом, MAU продукта, знание продуктов-спутников</v>
+      </c>
+      <c r="F30" s="372" t="str">
+        <v>окт.26</v>
+      </c>
+      <c r="G30" s="373" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" s="374" t="str">
+        <v>в работе</v>
+      </c>
+      <c r="I30" s="374"/>
+      <c r="J30" s="184"/>
+      <c r="K30" s="375" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="L30" s="375" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="M30" s="188" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="31">
+      <c r="A31" s="70" t="str">
+        <v>Сейфы_Воронка привлечения</v>
+      </c>
+      <c r="B31" s="369" t="str">
+        <v>Сейфы</v>
+      </c>
+      <c r="C31" s="327" t="str">
+        <v>Q42026</v>
+      </c>
+      <c r="D31" s="370" t="str">
+        <v>Воронка привлечения</v>
+      </c>
+      <c r="E31" s="371" t="str">
+        <v>Черновики в СБОЛ;
+Разработка CJM с воронками и процентами привлечения;
+Наличие Self-Service;
+Наличие бенчмарков - предоставить отчет по рынку</v>
+      </c>
+      <c r="F31" s="372" t="str">
+        <v>окт.26-дек.26</v>
+      </c>
+      <c r="G31" s="373" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="H31" s="374" t="str">
+        <v>в работе</v>
+      </c>
+      <c r="I31" s="374"/>
+      <c r="J31" s="184"/>
+      <c r="K31" s="375"/>
+      <c r="L31" s="375"/>
+      <c r="M31" s="188" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" r="32">
+      <c r="A32" s="70" t="str">
+        <v>Сейфы_Цели</v>
+      </c>
+      <c r="B32" s="369" t="str">
+        <v>Сейфы</v>
+      </c>
+      <c r="C32" s="327" t="str">
+        <v>Q42026</v>
+      </c>
+      <c r="D32" s="370" t="str">
+        <v>Цели</v>
+      </c>
+      <c r="E32" s="371" t="str">
+        <v>Цели уровня ЛЮ и ЛТ выведены на мониторинг и Прогноз по целям</v>
+      </c>
+      <c r="F32" s="372" t="str">
+        <v>дек.26</v>
+      </c>
+      <c r="G32" s="373" t="n">
+        <v>6</v>
+      </c>
+      <c r="H32" s="374" t="str">
+        <v>в работе</v>
+      </c>
+      <c r="I32" s="374"/>
+      <c r="J32" s="184"/>
+      <c r="K32" s="375"/>
+      <c r="L32" s="375"/>
+      <c r="M32" s="188" t="n">
+        <v>6</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="27">

</xml_diff>